<commit_message>
Remove project dates from memo and Disney files
</commit_message>
<xml_diff>
--- a/files/festival_forecast_model.xlsx
+++ b/files/festival_forecast_model.xlsx
@@ -70,7 +70,7 @@
     <t>Autumn Harvest Festival 2026 Attendance Forecast Model</t>
   </si>
   <si>
-    <t>WDPR Fall 2026 IE Case Study, Part 1. Built September 2026.</t>
+    <t>WDPR 2026 IE Case Study, Part 1. Built in 2026.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -271,7 +271,7 @@
     <t>-</t>
   </si>
   <si>
-    <t>Source: WDPR Fall 2026 IE Case Study, 'Historical Festival Attendance' table. 2021 may be COVID-affected; see Backtest and PDF for treatment.</t>
+    <t>Source: WDPR 2026 IE Case Study, 'Historical Festival Attendance' table. 2021 may be COVID-affected; see Backtest and PDF for treatment.</t>
   </si>
   <si>
     <t>Typical attendance distribution by weekend (seasonal index)</t>

</xml_diff>